<commit_message>
Use the sheet's em dash, not a hyphen, in added words
The first real word came back as "Small enclosed space - Cubiculo."
where every other row in the sheet reads "Evening meal - Cena." with an
em dash. The prompt was at fault: its rule said em dash while its worked
examples used a hyphen, because I had kept the file ASCII. The model
followed the example, as it should.

The examples now carry the character itself, and the rule points at them
rather than naming it. Belt and braces, meanings and notes are also
normalised on the way in: a hyphen or en dash with spaces around it is
the separator written wrongly and becomes an em dash, while a hyphen
inside a word -- open-plan -- has no spaces and is left alone.

The row already written was repaired in place, with a backup first, and
the app rebuilt: 1395 words, and Cubicle reads with the em dash.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I394"/>
+  <dimension ref="A1:I395"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col width="18.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -15979,7 +15979,33 @@
         </is>
       </c>
     </row>
-    <row r="395" ht="28.5" customHeight="1" s="22"/>
+    <row r="395" ht="28.5" customHeight="1" s="22">
+      <c r="A395" s="0" t="inlineStr">
+        <is>
+          <t>Cubicle</t>
+        </is>
+      </c>
+      <c r="B395" s="0" t="inlineStr">
+        <is>
+          <t>kiúbikel</t>
+        </is>
+      </c>
+      <c r="C395" s="0" t="inlineStr">
+        <is>
+          <t>Small enclosed space — Cubículo.</t>
+        </is>
+      </c>
+      <c r="D395" s="0" t="inlineStr">
+        <is>
+          <t>Lock the bathroom cubicle.</t>
+        </is>
+      </c>
+      <c r="I395" s="0" t="inlineStr">
+        <is>
+          <t>Common in British English for toilet stalls; also used for office partitions (open-plan cubicles).</t>
+        </is>
+      </c>
+    </row>
     <row r="396" ht="28.5" customHeight="1" s="22"/>
     <row r="397" ht="28.5" customHeight="1" s="22"/>
     <row r="398" ht="42.75" customHeight="1" s="22"/>

</xml_diff>

<commit_message>
Write the last fifty-five by hand
The key ran out of credit with fifty-five of the book's verbs still
unwritten, and waiting for billing is not a reason for him to be missing
a chapter. So they are written out here instead: the Spanish, the
pronunciation and the verb forms, in the conventions already in the
workbook -- "th" is z when it is voiceless and d when it is voiced,
w is u, and the stress carries a Spanish accent, so "see through"
is "sí zru" and "put up with" is "pút ap uith".

The book's own meaning and example are kept, as with every other row
from it; checked, all fifty-five.

All 321 verbs the book contained are now in the spreadsheet, and the app
has 1711 words.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I641"/>
+  <dimension ref="A1:I696"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col width="18.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -22865,6 +22865,1491 @@
       <c r="I641" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: take over — Present: takes over — Past: took over — Past participle: taken over. Separable: take something over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Pitch in</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>pich ín</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Help with a shared task — Echar una mano.</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Everyone pitched in to clean the house.</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: pitch in — Present: pitches in — Past: pitched in — Past participle: pitched in. Intransitive; not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Cheer up</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>chír ap</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Become happier — Animarse.</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Emma cheered up after hearing the good news.</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: cheer up — Present: cheers up — Past: cheered up — Past participle: cheered up. Separable: cheer someone up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Calm down</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>cálm daun</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Become less upset or angry — Calmarse.</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Tom calmed down after a few minutes.</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: calm down — Present: calms down — Past: calmed down — Past participle: calmed down. Separable: calm someone down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Brighten up</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>bráiten ap</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Become happier or more cheerful — Alegrarse.</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Sarah brightened up when she saw her friends.</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: brighten up — Present: brightens up — Past: brightened up — Past participle: brightened up. Also used of weather and of rooms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Open up</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>óupen ap</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Share your feelings with someone — Abrirse.</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Jack opened up to his best friend.</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: open up — Present: opens up — Past: opened up — Past participle: opened up. Intransitive in this sense: open up to someone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Bottle up</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>bótel ap</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Keep your feelings inside — Reprimir los sentimientos.</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Emma bottled up her emotions.</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: bottle up — Present: bottles up — Past: bottled up — Past participle: bottled up. Separable: bottle something up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Break down</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>bréik daun</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Lose control of your emotions — Derrumbarse.</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Sarah broke down in tears.</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: break down — Present: breaks down — Past: broke down — Past participle: broken down. Intransitive in this sense; of a machine it means to stop working.</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Hold back</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>jóuld bak</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Stop yourself from showing emotion — Contener.</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Jack held back his tears.</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: hold back — Present: holds back — Past: held back — Past participle: held back. Separable: hold something back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Bring down</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>bring dáun</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Make someone feel sad — Desanimar.</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>The bad news brought him down.</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: bring down — Present: brings down — Past: brought down — Past participle: brought down. Separable: bring someone down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Fall apart</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>fol apárt</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Become emotionally upset — Desmoronarse.</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Jack fell apart after the loss.</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: fall apart — Present: falls apart — Past: fell apart — Past participle: fallen apart. Intransitive; also used of things that break into pieces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Feel up to</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>fíl ap tu</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Feel able to do something — Sentirse capaz de.</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Tom didn't feel up to going out.</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: feel up to — Present: feels up to — Past: felt up to — Past participle: felt up to. Not separable. Followed by a noun or by -ing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Wear down</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>uér daun</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Make someone tired or stressed — Desgastar.</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>The long week wore him down.</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: wear down — Present: wears down — Past: wore down — Past participle: worn down. Separable: wear someone down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Ease up</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>ís ap</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Become less worried or tense — Relajarse.</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Sarah eased up after the test.</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: ease up — Present: eases up — Past: eased up — Past participle: eased up. Intransitive. Also said of rain or pressure letting up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Snap out of</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>snáp aut of</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Stop feeling sad or worried — Salir de un estado de ánimo.</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Emma snapped out of her bad mood.</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: snap out of — Present: snaps out of — Past: snapped out of — Past participle: snapped out of. Not separable. Often an imperative: snap out of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Lighten up</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>láiten ap</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Become less serious or worried — Tomárselo con calma.</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Jack lightened up after hearing the joke.</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: lighten up — Present: lightens up — Past: lightened up — Past participle: lightened up. Intransitive, and usually said as an instruction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Warm up to</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>uórm ap tu</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Gradually start liking someone — Agarrar confianza con.</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Sarah warmed up to her new neighbor.</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: warm up to — Present: warms up to — Past: warmed up to — Past participle: warmed up to. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Lean on</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>lín on</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Depend on someone for support — Apoyarse en.</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Emma leaned on her sister.</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: lean on — Present: leans on — Past: leaned on — Past participle: leaned on. Not separable. British English also uses leant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Well up</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>uél ap</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Fill with tears or strong emotion — Llenarse de lágrimas.</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Tears welled up in her eyes.</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: well up — Present: wells up — Past: welled up — Past participle: welled up. Intransitive. The subject is usually tears or a feeling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Come around</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>kam aráund</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Change your opinion or attitude — Cambiar de opinión.</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Tom came around after talking to her.</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: come around — Present: comes around — Past: came around — Past participle: come around. Intransitive. Also means to regain consciousness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Dwell on</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>duél on</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Keep thinking about something upsetting — Darle vueltas a.</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Emma dwelled on her mistake.</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: dwell on — Present: dwells on — Past: dwelled on — Past participle: dwelled on. Not separable. British English also uses dwelt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Shake off</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>shéik of</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Stop feeling something unpleasant — Quitarse de encima.</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Tom shook off his worries.</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: shake off — Present: shakes off — Past: shook off — Past participle: shaken off. Separable: shake something off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Hang on to</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>jáng on tu</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Keep a feeling or a memory — Aferrarse a.</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Emma hung on to her childhood memories.</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: hang on to — Present: hangs on to — Past: hung on to — Past participle: hung on to. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Sink in</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>sínk in</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Be fully understood — Asimilarse.</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>The news finally sank in.</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: sink in — Present: sinks in — Past: sank in — Past participle: sunk in. Intransitive. The subject is the news or the fact, not the person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Live through</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>lív zru</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Experience something difficult — Vivir algo difícil.</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Tom lived through a stressful year.</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: live through — Present: lives through — Past: lived through — Past participle: lived through. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Look down on</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>lúk daun on</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Think you are better than someone — Menospreciar.</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Jack looked down on his classmates.</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: look down on — Present: looks down on — Past: looked down on — Past participle: looked down on. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Beat yourself up</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>bít yorsélf ap</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Criticise yourself too much — Culparse demasiado.</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Emma beat herself up over the mistake.</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: beat yourself up — Present: beats himself up — Past: beat herself up — Past participle: beaten yourself up. The middle word changes with the person: beat myself up, beat himself up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Miss out on</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>mís aut on</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Lose the chance to experience something — Perderse algo.</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>Tom missed out on the trip.</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: miss out on — Present: misses out on — Past: missed out on — Past participle: missed out on. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Break into</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>bréik íntu</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Suddenly show an emotion — Echarse a.</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Emma broke into laughter.</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: break into — Present: breaks into — Past: broke into — Past participle: broken into. Not separable. Also means to enter a building by force.</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Get carried away</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>guét kárid auéi</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Become too excited or emotional — Dejarse llevar.</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Tom got carried away during the celebration.</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: get carried away — Present: gets carried away — Past: got carried away — Past participle: gotten carried away. A fixed expression; the three words stay together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Bottle out</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>bótel áut</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Lose courage and back out — Echarse atrás.</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Jack bottled out of giving the speech.</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: bottle out — Present: bottles out — Past: bottled out — Past participle: bottled out. Intransitive. British and informal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Fight back</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>fáit bak</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Stop yourself from showing emotion — Contener.</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Sarah fought back her tears.</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: fight back — Present: fights back — Past: fought back — Past participle: fought back. Separable in this sense. On its own it means to defend yourself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Clam up</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>klám ap</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Suddenly stop talking — Quedarse callado.</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Tom clammed up during the interview.</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: clam up — Present: clams up — Past: clammed up — Past participle: clammed up. Intransitive and informal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Bring about</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>bring abáut</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Cause something to happen — Provocar.</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>The new rule brought about positive changes.</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: bring about — Present: brings about — Past: brought about — Past participle: brought about. Separable, though the object usually follows the whole verb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Carry out</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>kári áut</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Complete a task or a plan — Llevar a cabo.</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>The students carried out the project successfully.</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: carry out — Present: carries out — Past: carried out — Past participle: carried out. Separable: carry it out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Come up with</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>kam ap uith</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Think of an idea or a solution — Ocurrírsele a uno.</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Sarah came up with a clever idea.</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: come up with — Present: comes up with — Past: came up with — Past participle: come up with. Not separable; all three words stay together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Turn out</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>tern áut</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Happen or develop in a particular way — Resultar.</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>The party turned out great.</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: turn out — Present: turns out — Past: turned out — Past participle: turned out. Intransitive in this sense. Often: it turned out that...</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Get away with</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>guét auéi uith</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Avoid punishment for something — Salirse con la suya.</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Jack got away with breaking the rules.</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: get away with — Present: gets away with — Past: got away with — Past participle: gotten away with. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Put up with</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>pút ap uith</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Tolerate something unpleasant — Aguantar.</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Sarah put up with the loud noise.</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: put up with — Present: puts up with — Past: put up with — Past participle: put up with. Not separable. The past looks the same as the base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Back out</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>bák áut</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Withdraw from an agreement or a plan — Echarse atrás.</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Jack backed out of the deal.</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: back out — Present: backs out — Past: backed out — Past participle: backed out. Intransitive: back out of something.</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Come up against</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>kam ap aguénst</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Face a difficulty — Toparse con.</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>The team came up against many problems.</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: come up against — Present: comes up against — Past: came up against — Past participle: come up against. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Drop out</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>dráp áut</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Leave a course before finishing — Abandonar los estudios.</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Jack dropped out of college.</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: drop out — Present: drops out — Past: dropped out — Past participle: dropped out. Intransitive: drop out of something.</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Get over with</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>guét óuver uith</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Finish something unpleasant — Terminar de una vez.</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Emma got the exam over with quickly.</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: get over with — Present: gets over with — Past: got over with — Past participle: gotten over with. The object goes in the middle: get it over with.</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Pull off</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>púl of</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Succeed in doing something difficult — Lograr.</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Sarah pulled off a great performance.</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: pull off — Present: pulls off — Past: pulled off — Past participle: pulled off. Separable: pull it off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Turn down</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>tern dáun</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Refuse an offer or a request — Rechazar.</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Emma turned down the job offer.</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: turn down — Present: turns down — Past: turned down — Past participle: turned down. Separable: turn it down. Also means to lower the volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Turn up</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>tern ap</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Appear or be found unexpectedly — Aparecer.</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>My keys turned up yesterday.</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: turn up — Present: turns up — Past: turned up — Past participle: turned up. Intransitive in this sense. Also means to raise the volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Work through</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>uérk zru</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Deal with a problem step by step — Resolver poco a poco.</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Sarah worked through her difficulties.</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: work through — Present: works through — Past: worked through — Past participle: worked through. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Write off</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>ráit of</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Consider something a loss — Dar por perdido.</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>The company wrote off the damaged equipment.</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: write off — Present: writes off — Past: wrote off — Past participle: written off. Separable: write it off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Pass up</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>pás ap</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Miss an opportunity by not taking it — Dejar pasar.</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Tom passed up a great offer.</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: pass up — Present: passes up — Past: passed up — Past participle: passed up. Separable: pass it up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Follow through</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>fólou zru</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Complete what you started — Cumplir hasta el final.</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Emma followed through on her promise.</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: follow through — Present: follows through — Past: followed through — Past participle: followed through. Not separable; usually follow through on something.</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Let down</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>lét daun</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Disappoint someone — Defraudar.</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Sarah let her team down.</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: let down — Present: lets down — Past: let down — Past participle: let down. Separable: let someone down. All the forms look the same.</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Call for</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>kol for</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Require something — Requerir.</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>The situation called for quick action.</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: call for — Present: calls for — Past: called for — Past participle: called for. Not separable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Rule out</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>rúl áut</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Eliminate a possibility — Descartar.</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>The doctor ruled out an infection.</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: rule out — Present: rules out — Past: ruled out — Past participle: ruled out. Separable: rule it out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Put down to</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>pút daun tu</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Explain something as caused by — Atribuir a.</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Tom put his success down to practice.</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: put down to — Present: puts down to — Past: put down to — Past participle: put down to. The object goes in the middle: put it down to luck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>See through</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>sí zru</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Recognise the truth about something — Calar.</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Emma saw through the excuse.</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: see through — Present: sees through — Past: saw through — Past participle: seen through. Not separable in this sense.</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Stand up for</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>stand ap for</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Defend someone or something — Defender.</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Jack stood up for his friend.</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>Irregular verb. Base: stand up for — Present: stands up for — Past: stood up for — Past participle: stood up for. Not separable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ask Google which model to use, and move on from a busy one
Two of the three model names written into this file had already been
withdrawn by the time a key was pasted in, and the third was overloaded.
Writing model names down was the mistake: the key is asked what it can
actually use now, and the best of those is taken -- newest, Flash,
full-fat, properly released. On this key that is Gemini 3.8 Flash, where
the list in the code would have reached nothing at all.

Busy is not broken either. The free tier is shared, so a spike is waited
out twice and then a different model is asked, rather than putting
"Gemini is busy" on screen while four models that would have answered sit
unused. Whichever answers is remembered, so it settles by itself on one
that is not congested.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -22869,1485 +22869,1485 @@
       </c>
     </row>
     <row r="642">
-      <c r="A642" t="inlineStr">
+      <c r="A642" s="0" t="inlineStr">
         <is>
           <t>Pitch in</t>
         </is>
       </c>
-      <c r="B642" t="inlineStr">
+      <c r="B642" s="0" t="inlineStr">
         <is>
           <t>pich ín</t>
         </is>
       </c>
-      <c r="C642" t="inlineStr">
+      <c r="C642" s="0" t="inlineStr">
         <is>
           <t>Help with a shared task — Echar una mano.</t>
         </is>
       </c>
-      <c r="D642" t="inlineStr">
+      <c r="D642" s="0" t="inlineStr">
         <is>
           <t>Everyone pitched in to clean the house.</t>
         </is>
       </c>
-      <c r="I642" t="inlineStr">
+      <c r="I642" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: pitch in — Present: pitches in — Past: pitched in — Past participle: pitched in. Intransitive; not separable.</t>
         </is>
       </c>
     </row>
     <row r="643">
-      <c r="A643" t="inlineStr">
+      <c r="A643" s="0" t="inlineStr">
         <is>
           <t>Cheer up</t>
         </is>
       </c>
-      <c r="B643" t="inlineStr">
+      <c r="B643" s="0" t="inlineStr">
         <is>
           <t>chír ap</t>
         </is>
       </c>
-      <c r="C643" t="inlineStr">
+      <c r="C643" s="0" t="inlineStr">
         <is>
           <t>Become happier — Animarse.</t>
         </is>
       </c>
-      <c r="D643" t="inlineStr">
+      <c r="D643" s="0" t="inlineStr">
         <is>
           <t>Emma cheered up after hearing the good news.</t>
         </is>
       </c>
-      <c r="I643" t="inlineStr">
+      <c r="I643" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: cheer up — Present: cheers up — Past: cheered up — Past participle: cheered up. Separable: cheer someone up.</t>
         </is>
       </c>
     </row>
     <row r="644">
-      <c r="A644" t="inlineStr">
+      <c r="A644" s="0" t="inlineStr">
         <is>
           <t>Calm down</t>
         </is>
       </c>
-      <c r="B644" t="inlineStr">
+      <c r="B644" s="0" t="inlineStr">
         <is>
           <t>cálm daun</t>
         </is>
       </c>
-      <c r="C644" t="inlineStr">
+      <c r="C644" s="0" t="inlineStr">
         <is>
           <t>Become less upset or angry — Calmarse.</t>
         </is>
       </c>
-      <c r="D644" t="inlineStr">
+      <c r="D644" s="0" t="inlineStr">
         <is>
           <t>Tom calmed down after a few minutes.</t>
         </is>
       </c>
-      <c r="I644" t="inlineStr">
+      <c r="I644" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: calm down — Present: calms down — Past: calmed down — Past participle: calmed down. Separable: calm someone down.</t>
         </is>
       </c>
     </row>
     <row r="645">
-      <c r="A645" t="inlineStr">
+      <c r="A645" s="0" t="inlineStr">
         <is>
           <t>Brighten up</t>
         </is>
       </c>
-      <c r="B645" t="inlineStr">
+      <c r="B645" s="0" t="inlineStr">
         <is>
           <t>bráiten ap</t>
         </is>
       </c>
-      <c r="C645" t="inlineStr">
+      <c r="C645" s="0" t="inlineStr">
         <is>
           <t>Become happier or more cheerful — Alegrarse.</t>
         </is>
       </c>
-      <c r="D645" t="inlineStr">
+      <c r="D645" s="0" t="inlineStr">
         <is>
           <t>Sarah brightened up when she saw her friends.</t>
         </is>
       </c>
-      <c r="I645" t="inlineStr">
+      <c r="I645" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: brighten up — Present: brightens up — Past: brightened up — Past participle: brightened up. Also used of weather and of rooms.</t>
         </is>
       </c>
     </row>
     <row r="646">
-      <c r="A646" t="inlineStr">
+      <c r="A646" s="0" t="inlineStr">
         <is>
           <t>Open up</t>
         </is>
       </c>
-      <c r="B646" t="inlineStr">
+      <c r="B646" s="0" t="inlineStr">
         <is>
           <t>óupen ap</t>
         </is>
       </c>
-      <c r="C646" t="inlineStr">
+      <c r="C646" s="0" t="inlineStr">
         <is>
           <t>Share your feelings with someone — Abrirse.</t>
         </is>
       </c>
-      <c r="D646" t="inlineStr">
+      <c r="D646" s="0" t="inlineStr">
         <is>
           <t>Jack opened up to his best friend.</t>
         </is>
       </c>
-      <c r="I646" t="inlineStr">
+      <c r="I646" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: open up — Present: opens up — Past: opened up — Past participle: opened up. Intransitive in this sense: open up to someone.</t>
         </is>
       </c>
     </row>
     <row r="647">
-      <c r="A647" t="inlineStr">
+      <c r="A647" s="0" t="inlineStr">
         <is>
           <t>Bottle up</t>
         </is>
       </c>
-      <c r="B647" t="inlineStr">
+      <c r="B647" s="0" t="inlineStr">
         <is>
           <t>bótel ap</t>
         </is>
       </c>
-      <c r="C647" t="inlineStr">
+      <c r="C647" s="0" t="inlineStr">
         <is>
           <t>Keep your feelings inside — Reprimir los sentimientos.</t>
         </is>
       </c>
-      <c r="D647" t="inlineStr">
+      <c r="D647" s="0" t="inlineStr">
         <is>
           <t>Emma bottled up her emotions.</t>
         </is>
       </c>
-      <c r="I647" t="inlineStr">
+      <c r="I647" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: bottle up — Present: bottles up — Past: bottled up — Past participle: bottled up. Separable: bottle something up.</t>
         </is>
       </c>
     </row>
     <row r="648">
-      <c r="A648" t="inlineStr">
+      <c r="A648" s="0" t="inlineStr">
         <is>
           <t>Break down</t>
         </is>
       </c>
-      <c r="B648" t="inlineStr">
+      <c r="B648" s="0" t="inlineStr">
         <is>
           <t>bréik daun</t>
         </is>
       </c>
-      <c r="C648" t="inlineStr">
+      <c r="C648" s="0" t="inlineStr">
         <is>
           <t>Lose control of your emotions — Derrumbarse.</t>
         </is>
       </c>
-      <c r="D648" t="inlineStr">
+      <c r="D648" s="0" t="inlineStr">
         <is>
           <t>Sarah broke down in tears.</t>
         </is>
       </c>
-      <c r="I648" t="inlineStr">
+      <c r="I648" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: break down — Present: breaks down — Past: broke down — Past participle: broken down. Intransitive in this sense; of a machine it means to stop working.</t>
         </is>
       </c>
     </row>
     <row r="649">
-      <c r="A649" t="inlineStr">
+      <c r="A649" s="0" t="inlineStr">
         <is>
           <t>Hold back</t>
         </is>
       </c>
-      <c r="B649" t="inlineStr">
+      <c r="B649" s="0" t="inlineStr">
         <is>
           <t>jóuld bak</t>
         </is>
       </c>
-      <c r="C649" t="inlineStr">
+      <c r="C649" s="0" t="inlineStr">
         <is>
           <t>Stop yourself from showing emotion — Contener.</t>
         </is>
       </c>
-      <c r="D649" t="inlineStr">
+      <c r="D649" s="0" t="inlineStr">
         <is>
           <t>Jack held back his tears.</t>
         </is>
       </c>
-      <c r="I649" t="inlineStr">
+      <c r="I649" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: hold back — Present: holds back — Past: held back — Past participle: held back. Separable: hold something back.</t>
         </is>
       </c>
     </row>
     <row r="650">
-      <c r="A650" t="inlineStr">
+      <c r="A650" s="0" t="inlineStr">
         <is>
           <t>Bring down</t>
         </is>
       </c>
-      <c r="B650" t="inlineStr">
+      <c r="B650" s="0" t="inlineStr">
         <is>
           <t>bring dáun</t>
         </is>
       </c>
-      <c r="C650" t="inlineStr">
+      <c r="C650" s="0" t="inlineStr">
         <is>
           <t>Make someone feel sad — Desanimar.</t>
         </is>
       </c>
-      <c r="D650" t="inlineStr">
+      <c r="D650" s="0" t="inlineStr">
         <is>
           <t>The bad news brought him down.</t>
         </is>
       </c>
-      <c r="I650" t="inlineStr">
+      <c r="I650" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: bring down — Present: brings down — Past: brought down — Past participle: brought down. Separable: bring someone down.</t>
         </is>
       </c>
     </row>
     <row r="651">
-      <c r="A651" t="inlineStr">
+      <c r="A651" s="0" t="inlineStr">
         <is>
           <t>Fall apart</t>
         </is>
       </c>
-      <c r="B651" t="inlineStr">
+      <c r="B651" s="0" t="inlineStr">
         <is>
           <t>fol apárt</t>
         </is>
       </c>
-      <c r="C651" t="inlineStr">
+      <c r="C651" s="0" t="inlineStr">
         <is>
           <t>Become emotionally upset — Desmoronarse.</t>
         </is>
       </c>
-      <c r="D651" t="inlineStr">
+      <c r="D651" s="0" t="inlineStr">
         <is>
           <t>Jack fell apart after the loss.</t>
         </is>
       </c>
-      <c r="I651" t="inlineStr">
+      <c r="I651" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: fall apart — Present: falls apart — Past: fell apart — Past participle: fallen apart. Intransitive; also used of things that break into pieces.</t>
         </is>
       </c>
     </row>
     <row r="652">
-      <c r="A652" t="inlineStr">
+      <c r="A652" s="0" t="inlineStr">
         <is>
           <t>Feel up to</t>
         </is>
       </c>
-      <c r="B652" t="inlineStr">
+      <c r="B652" s="0" t="inlineStr">
         <is>
           <t>fíl ap tu</t>
         </is>
       </c>
-      <c r="C652" t="inlineStr">
+      <c r="C652" s="0" t="inlineStr">
         <is>
           <t>Feel able to do something — Sentirse capaz de.</t>
         </is>
       </c>
-      <c r="D652" t="inlineStr">
+      <c r="D652" s="0" t="inlineStr">
         <is>
           <t>Tom didn't feel up to going out.</t>
         </is>
       </c>
-      <c r="I652" t="inlineStr">
+      <c r="I652" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: feel up to — Present: feels up to — Past: felt up to — Past participle: felt up to. Not separable. Followed by a noun or by -ing.</t>
         </is>
       </c>
     </row>
     <row r="653">
-      <c r="A653" t="inlineStr">
+      <c r="A653" s="0" t="inlineStr">
         <is>
           <t>Wear down</t>
         </is>
       </c>
-      <c r="B653" t="inlineStr">
+      <c r="B653" s="0" t="inlineStr">
         <is>
           <t>uér daun</t>
         </is>
       </c>
-      <c r="C653" t="inlineStr">
+      <c r="C653" s="0" t="inlineStr">
         <is>
           <t>Make someone tired or stressed — Desgastar.</t>
         </is>
       </c>
-      <c r="D653" t="inlineStr">
+      <c r="D653" s="0" t="inlineStr">
         <is>
           <t>The long week wore him down.</t>
         </is>
       </c>
-      <c r="I653" t="inlineStr">
+      <c r="I653" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: wear down — Present: wears down — Past: wore down — Past participle: worn down. Separable: wear someone down.</t>
         </is>
       </c>
     </row>
     <row r="654">
-      <c r="A654" t="inlineStr">
+      <c r="A654" s="0" t="inlineStr">
         <is>
           <t>Ease up</t>
         </is>
       </c>
-      <c r="B654" t="inlineStr">
+      <c r="B654" s="0" t="inlineStr">
         <is>
           <t>ís ap</t>
         </is>
       </c>
-      <c r="C654" t="inlineStr">
+      <c r="C654" s="0" t="inlineStr">
         <is>
           <t>Become less worried or tense — Relajarse.</t>
         </is>
       </c>
-      <c r="D654" t="inlineStr">
+      <c r="D654" s="0" t="inlineStr">
         <is>
           <t>Sarah eased up after the test.</t>
         </is>
       </c>
-      <c r="I654" t="inlineStr">
+      <c r="I654" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: ease up — Present: eases up — Past: eased up — Past participle: eased up. Intransitive. Also said of rain or pressure letting up.</t>
         </is>
       </c>
     </row>
     <row r="655">
-      <c r="A655" t="inlineStr">
+      <c r="A655" s="0" t="inlineStr">
         <is>
           <t>Snap out of</t>
         </is>
       </c>
-      <c r="B655" t="inlineStr">
+      <c r="B655" s="0" t="inlineStr">
         <is>
           <t>snáp aut of</t>
         </is>
       </c>
-      <c r="C655" t="inlineStr">
+      <c r="C655" s="0" t="inlineStr">
         <is>
           <t>Stop feeling sad or worried — Salir de un estado de ánimo.</t>
         </is>
       </c>
-      <c r="D655" t="inlineStr">
+      <c r="D655" s="0" t="inlineStr">
         <is>
           <t>Emma snapped out of her bad mood.</t>
         </is>
       </c>
-      <c r="I655" t="inlineStr">
+      <c r="I655" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: snap out of — Present: snaps out of — Past: snapped out of — Past participle: snapped out of. Not separable. Often an imperative: snap out of it.</t>
         </is>
       </c>
     </row>
     <row r="656">
-      <c r="A656" t="inlineStr">
+      <c r="A656" s="0" t="inlineStr">
         <is>
           <t>Lighten up</t>
         </is>
       </c>
-      <c r="B656" t="inlineStr">
+      <c r="B656" s="0" t="inlineStr">
         <is>
           <t>láiten ap</t>
         </is>
       </c>
-      <c r="C656" t="inlineStr">
+      <c r="C656" s="0" t="inlineStr">
         <is>
           <t>Become less serious or worried — Tomárselo con calma.</t>
         </is>
       </c>
-      <c r="D656" t="inlineStr">
+      <c r="D656" s="0" t="inlineStr">
         <is>
           <t>Jack lightened up after hearing the joke.</t>
         </is>
       </c>
-      <c r="I656" t="inlineStr">
+      <c r="I656" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: lighten up — Present: lightens up — Past: lightened up — Past participle: lightened up. Intransitive, and usually said as an instruction.</t>
         </is>
       </c>
     </row>
     <row r="657">
-      <c r="A657" t="inlineStr">
+      <c r="A657" s="0" t="inlineStr">
         <is>
           <t>Warm up to</t>
         </is>
       </c>
-      <c r="B657" t="inlineStr">
+      <c r="B657" s="0" t="inlineStr">
         <is>
           <t>uórm ap tu</t>
         </is>
       </c>
-      <c r="C657" t="inlineStr">
+      <c r="C657" s="0" t="inlineStr">
         <is>
           <t>Gradually start liking someone — Agarrar confianza con.</t>
         </is>
       </c>
-      <c r="D657" t="inlineStr">
+      <c r="D657" s="0" t="inlineStr">
         <is>
           <t>Sarah warmed up to her new neighbor.</t>
         </is>
       </c>
-      <c r="I657" t="inlineStr">
+      <c r="I657" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: warm up to — Present: warms up to — Past: warmed up to — Past participle: warmed up to. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="658">
-      <c r="A658" t="inlineStr">
+      <c r="A658" s="0" t="inlineStr">
         <is>
           <t>Lean on</t>
         </is>
       </c>
-      <c r="B658" t="inlineStr">
+      <c r="B658" s="0" t="inlineStr">
         <is>
           <t>lín on</t>
         </is>
       </c>
-      <c r="C658" t="inlineStr">
+      <c r="C658" s="0" t="inlineStr">
         <is>
           <t>Depend on someone for support — Apoyarse en.</t>
         </is>
       </c>
-      <c r="D658" t="inlineStr">
+      <c r="D658" s="0" t="inlineStr">
         <is>
           <t>Emma leaned on her sister.</t>
         </is>
       </c>
-      <c r="I658" t="inlineStr">
+      <c r="I658" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: lean on — Present: leans on — Past: leaned on — Past participle: leaned on. Not separable. British English also uses leant.</t>
         </is>
       </c>
     </row>
     <row r="659">
-      <c r="A659" t="inlineStr">
+      <c r="A659" s="0" t="inlineStr">
         <is>
           <t>Well up</t>
         </is>
       </c>
-      <c r="B659" t="inlineStr">
+      <c r="B659" s="0" t="inlineStr">
         <is>
           <t>uél ap</t>
         </is>
       </c>
-      <c r="C659" t="inlineStr">
+      <c r="C659" s="0" t="inlineStr">
         <is>
           <t>Fill with tears or strong emotion — Llenarse de lágrimas.</t>
         </is>
       </c>
-      <c r="D659" t="inlineStr">
+      <c r="D659" s="0" t="inlineStr">
         <is>
           <t>Tears welled up in her eyes.</t>
         </is>
       </c>
-      <c r="I659" t="inlineStr">
+      <c r="I659" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: well up — Present: wells up — Past: welled up — Past participle: welled up. Intransitive. The subject is usually tears or a feeling.</t>
         </is>
       </c>
     </row>
     <row r="660">
-      <c r="A660" t="inlineStr">
+      <c r="A660" s="0" t="inlineStr">
         <is>
           <t>Come around</t>
         </is>
       </c>
-      <c r="B660" t="inlineStr">
+      <c r="B660" s="0" t="inlineStr">
         <is>
           <t>kam aráund</t>
         </is>
       </c>
-      <c r="C660" t="inlineStr">
+      <c r="C660" s="0" t="inlineStr">
         <is>
           <t>Change your opinion or attitude — Cambiar de opinión.</t>
         </is>
       </c>
-      <c r="D660" t="inlineStr">
+      <c r="D660" s="0" t="inlineStr">
         <is>
           <t>Tom came around after talking to her.</t>
         </is>
       </c>
-      <c r="I660" t="inlineStr">
+      <c r="I660" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: come around — Present: comes around — Past: came around — Past participle: come around. Intransitive. Also means to regain consciousness.</t>
         </is>
       </c>
     </row>
     <row r="661">
-      <c r="A661" t="inlineStr">
+      <c r="A661" s="0" t="inlineStr">
         <is>
           <t>Dwell on</t>
         </is>
       </c>
-      <c r="B661" t="inlineStr">
+      <c r="B661" s="0" t="inlineStr">
         <is>
           <t>duél on</t>
         </is>
       </c>
-      <c r="C661" t="inlineStr">
+      <c r="C661" s="0" t="inlineStr">
         <is>
           <t>Keep thinking about something upsetting — Darle vueltas a.</t>
         </is>
       </c>
-      <c r="D661" t="inlineStr">
+      <c r="D661" s="0" t="inlineStr">
         <is>
           <t>Emma dwelled on her mistake.</t>
         </is>
       </c>
-      <c r="I661" t="inlineStr">
+      <c r="I661" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: dwell on — Present: dwells on — Past: dwelled on — Past participle: dwelled on. Not separable. British English also uses dwelt.</t>
         </is>
       </c>
     </row>
     <row r="662">
-      <c r="A662" t="inlineStr">
+      <c r="A662" s="0" t="inlineStr">
         <is>
           <t>Shake off</t>
         </is>
       </c>
-      <c r="B662" t="inlineStr">
+      <c r="B662" s="0" t="inlineStr">
         <is>
           <t>shéik of</t>
         </is>
       </c>
-      <c r="C662" t="inlineStr">
+      <c r="C662" s="0" t="inlineStr">
         <is>
           <t>Stop feeling something unpleasant — Quitarse de encima.</t>
         </is>
       </c>
-      <c r="D662" t="inlineStr">
+      <c r="D662" s="0" t="inlineStr">
         <is>
           <t>Tom shook off his worries.</t>
         </is>
       </c>
-      <c r="I662" t="inlineStr">
+      <c r="I662" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: shake off — Present: shakes off — Past: shook off — Past participle: shaken off. Separable: shake something off.</t>
         </is>
       </c>
     </row>
     <row r="663">
-      <c r="A663" t="inlineStr">
+      <c r="A663" s="0" t="inlineStr">
         <is>
           <t>Hang on to</t>
         </is>
       </c>
-      <c r="B663" t="inlineStr">
+      <c r="B663" s="0" t="inlineStr">
         <is>
           <t>jáng on tu</t>
         </is>
       </c>
-      <c r="C663" t="inlineStr">
+      <c r="C663" s="0" t="inlineStr">
         <is>
           <t>Keep a feeling or a memory — Aferrarse a.</t>
         </is>
       </c>
-      <c r="D663" t="inlineStr">
+      <c r="D663" s="0" t="inlineStr">
         <is>
           <t>Emma hung on to her childhood memories.</t>
         </is>
       </c>
-      <c r="I663" t="inlineStr">
+      <c r="I663" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: hang on to — Present: hangs on to — Past: hung on to — Past participle: hung on to. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="664">
-      <c r="A664" t="inlineStr">
+      <c r="A664" s="0" t="inlineStr">
         <is>
           <t>Sink in</t>
         </is>
       </c>
-      <c r="B664" t="inlineStr">
+      <c r="B664" s="0" t="inlineStr">
         <is>
           <t>sínk in</t>
         </is>
       </c>
-      <c r="C664" t="inlineStr">
+      <c r="C664" s="0" t="inlineStr">
         <is>
           <t>Be fully understood — Asimilarse.</t>
         </is>
       </c>
-      <c r="D664" t="inlineStr">
+      <c r="D664" s="0" t="inlineStr">
         <is>
           <t>The news finally sank in.</t>
         </is>
       </c>
-      <c r="I664" t="inlineStr">
+      <c r="I664" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: sink in — Present: sinks in — Past: sank in — Past participle: sunk in. Intransitive. The subject is the news or the fact, not the person.</t>
         </is>
       </c>
     </row>
     <row r="665">
-      <c r="A665" t="inlineStr">
+      <c r="A665" s="0" t="inlineStr">
         <is>
           <t>Live through</t>
         </is>
       </c>
-      <c r="B665" t="inlineStr">
+      <c r="B665" s="0" t="inlineStr">
         <is>
           <t>lív zru</t>
         </is>
       </c>
-      <c r="C665" t="inlineStr">
+      <c r="C665" s="0" t="inlineStr">
         <is>
           <t>Experience something difficult — Vivir algo difícil.</t>
         </is>
       </c>
-      <c r="D665" t="inlineStr">
+      <c r="D665" s="0" t="inlineStr">
         <is>
           <t>Tom lived through a stressful year.</t>
         </is>
       </c>
-      <c r="I665" t="inlineStr">
+      <c r="I665" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: live through — Present: lives through — Past: lived through — Past participle: lived through. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="666">
-      <c r="A666" t="inlineStr">
+      <c r="A666" s="0" t="inlineStr">
         <is>
           <t>Look down on</t>
         </is>
       </c>
-      <c r="B666" t="inlineStr">
+      <c r="B666" s="0" t="inlineStr">
         <is>
           <t>lúk daun on</t>
         </is>
       </c>
-      <c r="C666" t="inlineStr">
+      <c r="C666" s="0" t="inlineStr">
         <is>
           <t>Think you are better than someone — Menospreciar.</t>
         </is>
       </c>
-      <c r="D666" t="inlineStr">
+      <c r="D666" s="0" t="inlineStr">
         <is>
           <t>Jack looked down on his classmates.</t>
         </is>
       </c>
-      <c r="I666" t="inlineStr">
+      <c r="I666" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: look down on — Present: looks down on — Past: looked down on — Past participle: looked down on. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="667">
-      <c r="A667" t="inlineStr">
+      <c r="A667" s="0" t="inlineStr">
         <is>
           <t>Beat yourself up</t>
         </is>
       </c>
-      <c r="B667" t="inlineStr">
+      <c r="B667" s="0" t="inlineStr">
         <is>
           <t>bít yorsélf ap</t>
         </is>
       </c>
-      <c r="C667" t="inlineStr">
+      <c r="C667" s="0" t="inlineStr">
         <is>
           <t>Criticise yourself too much — Culparse demasiado.</t>
         </is>
       </c>
-      <c r="D667" t="inlineStr">
+      <c r="D667" s="0" t="inlineStr">
         <is>
           <t>Emma beat herself up over the mistake.</t>
         </is>
       </c>
-      <c r="I667" t="inlineStr">
+      <c r="I667" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: beat yourself up — Present: beats himself up — Past: beat herself up — Past participle: beaten yourself up. The middle word changes with the person: beat myself up, beat himself up.</t>
         </is>
       </c>
     </row>
     <row r="668">
-      <c r="A668" t="inlineStr">
+      <c r="A668" s="0" t="inlineStr">
         <is>
           <t>Miss out on</t>
         </is>
       </c>
-      <c r="B668" t="inlineStr">
+      <c r="B668" s="0" t="inlineStr">
         <is>
           <t>mís aut on</t>
         </is>
       </c>
-      <c r="C668" t="inlineStr">
+      <c r="C668" s="0" t="inlineStr">
         <is>
           <t>Lose the chance to experience something — Perderse algo.</t>
         </is>
       </c>
-      <c r="D668" t="inlineStr">
+      <c r="D668" s="0" t="inlineStr">
         <is>
           <t>Tom missed out on the trip.</t>
         </is>
       </c>
-      <c r="I668" t="inlineStr">
+      <c r="I668" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: miss out on — Present: misses out on — Past: missed out on — Past participle: missed out on. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="669">
-      <c r="A669" t="inlineStr">
+      <c r="A669" s="0" t="inlineStr">
         <is>
           <t>Break into</t>
         </is>
       </c>
-      <c r="B669" t="inlineStr">
+      <c r="B669" s="0" t="inlineStr">
         <is>
           <t>bréik íntu</t>
         </is>
       </c>
-      <c r="C669" t="inlineStr">
+      <c r="C669" s="0" t="inlineStr">
         <is>
           <t>Suddenly show an emotion — Echarse a.</t>
         </is>
       </c>
-      <c r="D669" t="inlineStr">
+      <c r="D669" s="0" t="inlineStr">
         <is>
           <t>Emma broke into laughter.</t>
         </is>
       </c>
-      <c r="I669" t="inlineStr">
+      <c r="I669" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: break into — Present: breaks into — Past: broke into — Past participle: broken into. Not separable. Also means to enter a building by force.</t>
         </is>
       </c>
     </row>
     <row r="670">
-      <c r="A670" t="inlineStr">
+      <c r="A670" s="0" t="inlineStr">
         <is>
           <t>Get carried away</t>
         </is>
       </c>
-      <c r="B670" t="inlineStr">
+      <c r="B670" s="0" t="inlineStr">
         <is>
           <t>guét kárid auéi</t>
         </is>
       </c>
-      <c r="C670" t="inlineStr">
+      <c r="C670" s="0" t="inlineStr">
         <is>
           <t>Become too excited or emotional — Dejarse llevar.</t>
         </is>
       </c>
-      <c r="D670" t="inlineStr">
+      <c r="D670" s="0" t="inlineStr">
         <is>
           <t>Tom got carried away during the celebration.</t>
         </is>
       </c>
-      <c r="I670" t="inlineStr">
+      <c r="I670" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: get carried away — Present: gets carried away — Past: got carried away — Past participle: gotten carried away. A fixed expression; the three words stay together.</t>
         </is>
       </c>
     </row>
     <row r="671">
-      <c r="A671" t="inlineStr">
+      <c r="A671" s="0" t="inlineStr">
         <is>
           <t>Bottle out</t>
         </is>
       </c>
-      <c r="B671" t="inlineStr">
+      <c r="B671" s="0" t="inlineStr">
         <is>
           <t>bótel áut</t>
         </is>
       </c>
-      <c r="C671" t="inlineStr">
+      <c r="C671" s="0" t="inlineStr">
         <is>
           <t>Lose courage and back out — Echarse atrás.</t>
         </is>
       </c>
-      <c r="D671" t="inlineStr">
+      <c r="D671" s="0" t="inlineStr">
         <is>
           <t>Jack bottled out of giving the speech.</t>
         </is>
       </c>
-      <c r="I671" t="inlineStr">
+      <c r="I671" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: bottle out — Present: bottles out — Past: bottled out — Past participle: bottled out. Intransitive. British and informal.</t>
         </is>
       </c>
     </row>
     <row r="672">
-      <c r="A672" t="inlineStr">
+      <c r="A672" s="0" t="inlineStr">
         <is>
           <t>Fight back</t>
         </is>
       </c>
-      <c r="B672" t="inlineStr">
+      <c r="B672" s="0" t="inlineStr">
         <is>
           <t>fáit bak</t>
         </is>
       </c>
-      <c r="C672" t="inlineStr">
+      <c r="C672" s="0" t="inlineStr">
         <is>
           <t>Stop yourself from showing emotion — Contener.</t>
         </is>
       </c>
-      <c r="D672" t="inlineStr">
+      <c r="D672" s="0" t="inlineStr">
         <is>
           <t>Sarah fought back her tears.</t>
         </is>
       </c>
-      <c r="I672" t="inlineStr">
+      <c r="I672" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: fight back — Present: fights back — Past: fought back — Past participle: fought back. Separable in this sense. On its own it means to defend yourself.</t>
         </is>
       </c>
     </row>
     <row r="673">
-      <c r="A673" t="inlineStr">
+      <c r="A673" s="0" t="inlineStr">
         <is>
           <t>Clam up</t>
         </is>
       </c>
-      <c r="B673" t="inlineStr">
+      <c r="B673" s="0" t="inlineStr">
         <is>
           <t>klám ap</t>
         </is>
       </c>
-      <c r="C673" t="inlineStr">
+      <c r="C673" s="0" t="inlineStr">
         <is>
           <t>Suddenly stop talking — Quedarse callado.</t>
         </is>
       </c>
-      <c r="D673" t="inlineStr">
+      <c r="D673" s="0" t="inlineStr">
         <is>
           <t>Tom clammed up during the interview.</t>
         </is>
       </c>
-      <c r="I673" t="inlineStr">
+      <c r="I673" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: clam up — Present: clams up — Past: clammed up — Past participle: clammed up. Intransitive and informal.</t>
         </is>
       </c>
     </row>
     <row r="674">
-      <c r="A674" t="inlineStr">
+      <c r="A674" s="0" t="inlineStr">
         <is>
           <t>Bring about</t>
         </is>
       </c>
-      <c r="B674" t="inlineStr">
+      <c r="B674" s="0" t="inlineStr">
         <is>
           <t>bring abáut</t>
         </is>
       </c>
-      <c r="C674" t="inlineStr">
+      <c r="C674" s="0" t="inlineStr">
         <is>
           <t>Cause something to happen — Provocar.</t>
         </is>
       </c>
-      <c r="D674" t="inlineStr">
+      <c r="D674" s="0" t="inlineStr">
         <is>
           <t>The new rule brought about positive changes.</t>
         </is>
       </c>
-      <c r="I674" t="inlineStr">
+      <c r="I674" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: bring about — Present: brings about — Past: brought about — Past participle: brought about. Separable, though the object usually follows the whole verb.</t>
         </is>
       </c>
     </row>
     <row r="675">
-      <c r="A675" t="inlineStr">
+      <c r="A675" s="0" t="inlineStr">
         <is>
           <t>Carry out</t>
         </is>
       </c>
-      <c r="B675" t="inlineStr">
+      <c r="B675" s="0" t="inlineStr">
         <is>
           <t>kári áut</t>
         </is>
       </c>
-      <c r="C675" t="inlineStr">
+      <c r="C675" s="0" t="inlineStr">
         <is>
           <t>Complete a task or a plan — Llevar a cabo.</t>
         </is>
       </c>
-      <c r="D675" t="inlineStr">
+      <c r="D675" s="0" t="inlineStr">
         <is>
           <t>The students carried out the project successfully.</t>
         </is>
       </c>
-      <c r="I675" t="inlineStr">
+      <c r="I675" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: carry out — Present: carries out — Past: carried out — Past participle: carried out. Separable: carry it out.</t>
         </is>
       </c>
     </row>
     <row r="676">
-      <c r="A676" t="inlineStr">
+      <c r="A676" s="0" t="inlineStr">
         <is>
           <t>Come up with</t>
         </is>
       </c>
-      <c r="B676" t="inlineStr">
+      <c r="B676" s="0" t="inlineStr">
         <is>
           <t>kam ap uith</t>
         </is>
       </c>
-      <c r="C676" t="inlineStr">
+      <c r="C676" s="0" t="inlineStr">
         <is>
           <t>Think of an idea or a solution — Ocurrírsele a uno.</t>
         </is>
       </c>
-      <c r="D676" t="inlineStr">
+      <c r="D676" s="0" t="inlineStr">
         <is>
           <t>Sarah came up with a clever idea.</t>
         </is>
       </c>
-      <c r="I676" t="inlineStr">
+      <c r="I676" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: come up with — Present: comes up with — Past: came up with — Past participle: come up with. Not separable; all three words stay together.</t>
         </is>
       </c>
     </row>
     <row r="677">
-      <c r="A677" t="inlineStr">
+      <c r="A677" s="0" t="inlineStr">
         <is>
           <t>Turn out</t>
         </is>
       </c>
-      <c r="B677" t="inlineStr">
+      <c r="B677" s="0" t="inlineStr">
         <is>
           <t>tern áut</t>
         </is>
       </c>
-      <c r="C677" t="inlineStr">
+      <c r="C677" s="0" t="inlineStr">
         <is>
           <t>Happen or develop in a particular way — Resultar.</t>
         </is>
       </c>
-      <c r="D677" t="inlineStr">
+      <c r="D677" s="0" t="inlineStr">
         <is>
           <t>The party turned out great.</t>
         </is>
       </c>
-      <c r="I677" t="inlineStr">
+      <c r="I677" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: turn out — Present: turns out — Past: turned out — Past participle: turned out. Intransitive in this sense. Often: it turned out that...</t>
         </is>
       </c>
     </row>
     <row r="678">
-      <c r="A678" t="inlineStr">
+      <c r="A678" s="0" t="inlineStr">
         <is>
           <t>Get away with</t>
         </is>
       </c>
-      <c r="B678" t="inlineStr">
+      <c r="B678" s="0" t="inlineStr">
         <is>
           <t>guét auéi uith</t>
         </is>
       </c>
-      <c r="C678" t="inlineStr">
+      <c r="C678" s="0" t="inlineStr">
         <is>
           <t>Avoid punishment for something — Salirse con la suya.</t>
         </is>
       </c>
-      <c r="D678" t="inlineStr">
+      <c r="D678" s="0" t="inlineStr">
         <is>
           <t>Jack got away with breaking the rules.</t>
         </is>
       </c>
-      <c r="I678" t="inlineStr">
+      <c r="I678" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: get away with — Present: gets away with — Past: got away with — Past participle: gotten away with. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="679">
-      <c r="A679" t="inlineStr">
+      <c r="A679" s="0" t="inlineStr">
         <is>
           <t>Put up with</t>
         </is>
       </c>
-      <c r="B679" t="inlineStr">
+      <c r="B679" s="0" t="inlineStr">
         <is>
           <t>pút ap uith</t>
         </is>
       </c>
-      <c r="C679" t="inlineStr">
+      <c r="C679" s="0" t="inlineStr">
         <is>
           <t>Tolerate something unpleasant — Aguantar.</t>
         </is>
       </c>
-      <c r="D679" t="inlineStr">
+      <c r="D679" s="0" t="inlineStr">
         <is>
           <t>Sarah put up with the loud noise.</t>
         </is>
       </c>
-      <c r="I679" t="inlineStr">
+      <c r="I679" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: put up with — Present: puts up with — Past: put up with — Past participle: put up with. Not separable. The past looks the same as the base.</t>
         </is>
       </c>
     </row>
     <row r="680">
-      <c r="A680" t="inlineStr">
+      <c r="A680" s="0" t="inlineStr">
         <is>
           <t>Back out</t>
         </is>
       </c>
-      <c r="B680" t="inlineStr">
+      <c r="B680" s="0" t="inlineStr">
         <is>
           <t>bák áut</t>
         </is>
       </c>
-      <c r="C680" t="inlineStr">
+      <c r="C680" s="0" t="inlineStr">
         <is>
           <t>Withdraw from an agreement or a plan — Echarse atrás.</t>
         </is>
       </c>
-      <c r="D680" t="inlineStr">
+      <c r="D680" s="0" t="inlineStr">
         <is>
           <t>Jack backed out of the deal.</t>
         </is>
       </c>
-      <c r="I680" t="inlineStr">
+      <c r="I680" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: back out — Present: backs out — Past: backed out — Past participle: backed out. Intransitive: back out of something.</t>
         </is>
       </c>
     </row>
     <row r="681">
-      <c r="A681" t="inlineStr">
+      <c r="A681" s="0" t="inlineStr">
         <is>
           <t>Come up against</t>
         </is>
       </c>
-      <c r="B681" t="inlineStr">
+      <c r="B681" s="0" t="inlineStr">
         <is>
           <t>kam ap aguénst</t>
         </is>
       </c>
-      <c r="C681" t="inlineStr">
+      <c r="C681" s="0" t="inlineStr">
         <is>
           <t>Face a difficulty — Toparse con.</t>
         </is>
       </c>
-      <c r="D681" t="inlineStr">
+      <c r="D681" s="0" t="inlineStr">
         <is>
           <t>The team came up against many problems.</t>
         </is>
       </c>
-      <c r="I681" t="inlineStr">
+      <c r="I681" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: come up against — Present: comes up against — Past: came up against — Past participle: come up against. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="682">
-      <c r="A682" t="inlineStr">
+      <c r="A682" s="0" t="inlineStr">
         <is>
           <t>Drop out</t>
         </is>
       </c>
-      <c r="B682" t="inlineStr">
+      <c r="B682" s="0" t="inlineStr">
         <is>
           <t>dráp áut</t>
         </is>
       </c>
-      <c r="C682" t="inlineStr">
+      <c r="C682" s="0" t="inlineStr">
         <is>
           <t>Leave a course before finishing — Abandonar los estudios.</t>
         </is>
       </c>
-      <c r="D682" t="inlineStr">
+      <c r="D682" s="0" t="inlineStr">
         <is>
           <t>Jack dropped out of college.</t>
         </is>
       </c>
-      <c r="I682" t="inlineStr">
+      <c r="I682" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: drop out — Present: drops out — Past: dropped out — Past participle: dropped out. Intransitive: drop out of something.</t>
         </is>
       </c>
     </row>
     <row r="683">
-      <c r="A683" t="inlineStr">
+      <c r="A683" s="0" t="inlineStr">
         <is>
           <t>Get over with</t>
         </is>
       </c>
-      <c r="B683" t="inlineStr">
+      <c r="B683" s="0" t="inlineStr">
         <is>
           <t>guét óuver uith</t>
         </is>
       </c>
-      <c r="C683" t="inlineStr">
+      <c r="C683" s="0" t="inlineStr">
         <is>
           <t>Finish something unpleasant — Terminar de una vez.</t>
         </is>
       </c>
-      <c r="D683" t="inlineStr">
+      <c r="D683" s="0" t="inlineStr">
         <is>
           <t>Emma got the exam over with quickly.</t>
         </is>
       </c>
-      <c r="I683" t="inlineStr">
+      <c r="I683" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: get over with — Present: gets over with — Past: got over with — Past participle: gotten over with. The object goes in the middle: get it over with.</t>
         </is>
       </c>
     </row>
     <row r="684">
-      <c r="A684" t="inlineStr">
+      <c r="A684" s="0" t="inlineStr">
         <is>
           <t>Pull off</t>
         </is>
       </c>
-      <c r="B684" t="inlineStr">
+      <c r="B684" s="0" t="inlineStr">
         <is>
           <t>púl of</t>
         </is>
       </c>
-      <c r="C684" t="inlineStr">
+      <c r="C684" s="0" t="inlineStr">
         <is>
           <t>Succeed in doing something difficult — Lograr.</t>
         </is>
       </c>
-      <c r="D684" t="inlineStr">
+      <c r="D684" s="0" t="inlineStr">
         <is>
           <t>Sarah pulled off a great performance.</t>
         </is>
       </c>
-      <c r="I684" t="inlineStr">
+      <c r="I684" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: pull off — Present: pulls off — Past: pulled off — Past participle: pulled off. Separable: pull it off.</t>
         </is>
       </c>
     </row>
     <row r="685">
-      <c r="A685" t="inlineStr">
+      <c r="A685" s="0" t="inlineStr">
         <is>
           <t>Turn down</t>
         </is>
       </c>
-      <c r="B685" t="inlineStr">
+      <c r="B685" s="0" t="inlineStr">
         <is>
           <t>tern dáun</t>
         </is>
       </c>
-      <c r="C685" t="inlineStr">
+      <c r="C685" s="0" t="inlineStr">
         <is>
           <t>Refuse an offer or a request — Rechazar.</t>
         </is>
       </c>
-      <c r="D685" t="inlineStr">
+      <c r="D685" s="0" t="inlineStr">
         <is>
           <t>Emma turned down the job offer.</t>
         </is>
       </c>
-      <c r="I685" t="inlineStr">
+      <c r="I685" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: turn down — Present: turns down — Past: turned down — Past participle: turned down. Separable: turn it down. Also means to lower the volume.</t>
         </is>
       </c>
     </row>
     <row r="686">
-      <c r="A686" t="inlineStr">
+      <c r="A686" s="0" t="inlineStr">
         <is>
           <t>Turn up</t>
         </is>
       </c>
-      <c r="B686" t="inlineStr">
+      <c r="B686" s="0" t="inlineStr">
         <is>
           <t>tern ap</t>
         </is>
       </c>
-      <c r="C686" t="inlineStr">
+      <c r="C686" s="0" t="inlineStr">
         <is>
           <t>Appear or be found unexpectedly — Aparecer.</t>
         </is>
       </c>
-      <c r="D686" t="inlineStr">
+      <c r="D686" s="0" t="inlineStr">
         <is>
           <t>My keys turned up yesterday.</t>
         </is>
       </c>
-      <c r="I686" t="inlineStr">
+      <c r="I686" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: turn up — Present: turns up — Past: turned up — Past participle: turned up. Intransitive in this sense. Also means to raise the volume.</t>
         </is>
       </c>
     </row>
     <row r="687">
-      <c r="A687" t="inlineStr">
+      <c r="A687" s="0" t="inlineStr">
         <is>
           <t>Work through</t>
         </is>
       </c>
-      <c r="B687" t="inlineStr">
+      <c r="B687" s="0" t="inlineStr">
         <is>
           <t>uérk zru</t>
         </is>
       </c>
-      <c r="C687" t="inlineStr">
+      <c r="C687" s="0" t="inlineStr">
         <is>
           <t>Deal with a problem step by step — Resolver poco a poco.</t>
         </is>
       </c>
-      <c r="D687" t="inlineStr">
+      <c r="D687" s="0" t="inlineStr">
         <is>
           <t>Sarah worked through her difficulties.</t>
         </is>
       </c>
-      <c r="I687" t="inlineStr">
+      <c r="I687" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: work through — Present: works through — Past: worked through — Past participle: worked through. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="688">
-      <c r="A688" t="inlineStr">
+      <c r="A688" s="0" t="inlineStr">
         <is>
           <t>Write off</t>
         </is>
       </c>
-      <c r="B688" t="inlineStr">
+      <c r="B688" s="0" t="inlineStr">
         <is>
           <t>ráit of</t>
         </is>
       </c>
-      <c r="C688" t="inlineStr">
+      <c r="C688" s="0" t="inlineStr">
         <is>
           <t>Consider something a loss — Dar por perdido.</t>
         </is>
       </c>
-      <c r="D688" t="inlineStr">
+      <c r="D688" s="0" t="inlineStr">
         <is>
           <t>The company wrote off the damaged equipment.</t>
         </is>
       </c>
-      <c r="I688" t="inlineStr">
+      <c r="I688" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: write off — Present: writes off — Past: wrote off — Past participle: written off. Separable: write it off.</t>
         </is>
       </c>
     </row>
     <row r="689">
-      <c r="A689" t="inlineStr">
+      <c r="A689" s="0" t="inlineStr">
         <is>
           <t>Pass up</t>
         </is>
       </c>
-      <c r="B689" t="inlineStr">
+      <c r="B689" s="0" t="inlineStr">
         <is>
           <t>pás ap</t>
         </is>
       </c>
-      <c r="C689" t="inlineStr">
+      <c r="C689" s="0" t="inlineStr">
         <is>
           <t>Miss an opportunity by not taking it — Dejar pasar.</t>
         </is>
       </c>
-      <c r="D689" t="inlineStr">
+      <c r="D689" s="0" t="inlineStr">
         <is>
           <t>Tom passed up a great offer.</t>
         </is>
       </c>
-      <c r="I689" t="inlineStr">
+      <c r="I689" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: pass up — Present: passes up — Past: passed up — Past participle: passed up. Separable: pass it up.</t>
         </is>
       </c>
     </row>
     <row r="690">
-      <c r="A690" t="inlineStr">
+      <c r="A690" s="0" t="inlineStr">
         <is>
           <t>Follow through</t>
         </is>
       </c>
-      <c r="B690" t="inlineStr">
+      <c r="B690" s="0" t="inlineStr">
         <is>
           <t>fólou zru</t>
         </is>
       </c>
-      <c r="C690" t="inlineStr">
+      <c r="C690" s="0" t="inlineStr">
         <is>
           <t>Complete what you started — Cumplir hasta el final.</t>
         </is>
       </c>
-      <c r="D690" t="inlineStr">
+      <c r="D690" s="0" t="inlineStr">
         <is>
           <t>Emma followed through on her promise.</t>
         </is>
       </c>
-      <c r="I690" t="inlineStr">
+      <c r="I690" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: follow through — Present: follows through — Past: followed through — Past participle: followed through. Not separable; usually follow through on something.</t>
         </is>
       </c>
     </row>
     <row r="691">
-      <c r="A691" t="inlineStr">
+      <c r="A691" s="0" t="inlineStr">
         <is>
           <t>Let down</t>
         </is>
       </c>
-      <c r="B691" t="inlineStr">
+      <c r="B691" s="0" t="inlineStr">
         <is>
           <t>lét daun</t>
         </is>
       </c>
-      <c r="C691" t="inlineStr">
+      <c r="C691" s="0" t="inlineStr">
         <is>
           <t>Disappoint someone — Defraudar.</t>
         </is>
       </c>
-      <c r="D691" t="inlineStr">
+      <c r="D691" s="0" t="inlineStr">
         <is>
           <t>Sarah let her team down.</t>
         </is>
       </c>
-      <c r="I691" t="inlineStr">
+      <c r="I691" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: let down — Present: lets down — Past: let down — Past participle: let down. Separable: let someone down. All the forms look the same.</t>
         </is>
       </c>
     </row>
     <row r="692">
-      <c r="A692" t="inlineStr">
+      <c r="A692" s="0" t="inlineStr">
         <is>
           <t>Call for</t>
         </is>
       </c>
-      <c r="B692" t="inlineStr">
+      <c r="B692" s="0" t="inlineStr">
         <is>
           <t>kol for</t>
         </is>
       </c>
-      <c r="C692" t="inlineStr">
+      <c r="C692" s="0" t="inlineStr">
         <is>
           <t>Require something — Requerir.</t>
         </is>
       </c>
-      <c r="D692" t="inlineStr">
+      <c r="D692" s="0" t="inlineStr">
         <is>
           <t>The situation called for quick action.</t>
         </is>
       </c>
-      <c r="I692" t="inlineStr">
+      <c r="I692" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: call for — Present: calls for — Past: called for — Past participle: called for. Not separable.</t>
         </is>
       </c>
     </row>
     <row r="693">
-      <c r="A693" t="inlineStr">
+      <c r="A693" s="0" t="inlineStr">
         <is>
           <t>Rule out</t>
         </is>
       </c>
-      <c r="B693" t="inlineStr">
+      <c r="B693" s="0" t="inlineStr">
         <is>
           <t>rúl áut</t>
         </is>
       </c>
-      <c r="C693" t="inlineStr">
+      <c r="C693" s="0" t="inlineStr">
         <is>
           <t>Eliminate a possibility — Descartar.</t>
         </is>
       </c>
-      <c r="D693" t="inlineStr">
+      <c r="D693" s="0" t="inlineStr">
         <is>
           <t>The doctor ruled out an infection.</t>
         </is>
       </c>
-      <c r="I693" t="inlineStr">
+      <c r="I693" s="0" t="inlineStr">
         <is>
           <t>Regular verb. Base: rule out — Present: rules out — Past: ruled out — Past participle: ruled out. Separable: rule it out.</t>
         </is>
       </c>
     </row>
     <row r="694">
-      <c r="A694" t="inlineStr">
+      <c r="A694" s="0" t="inlineStr">
         <is>
           <t>Put down to</t>
         </is>
       </c>
-      <c r="B694" t="inlineStr">
+      <c r="B694" s="0" t="inlineStr">
         <is>
           <t>pút daun tu</t>
         </is>
       </c>
-      <c r="C694" t="inlineStr">
+      <c r="C694" s="0" t="inlineStr">
         <is>
           <t>Explain something as caused by — Atribuir a.</t>
         </is>
       </c>
-      <c r="D694" t="inlineStr">
+      <c r="D694" s="0" t="inlineStr">
         <is>
           <t>Tom put his success down to practice.</t>
         </is>
       </c>
-      <c r="I694" t="inlineStr">
+      <c r="I694" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: put down to — Present: puts down to — Past: put down to — Past participle: put down to. The object goes in the middle: put it down to luck.</t>
         </is>
       </c>
     </row>
     <row r="695">
-      <c r="A695" t="inlineStr">
+      <c r="A695" s="0" t="inlineStr">
         <is>
           <t>See through</t>
         </is>
       </c>
-      <c r="B695" t="inlineStr">
+      <c r="B695" s="0" t="inlineStr">
         <is>
           <t>sí zru</t>
         </is>
       </c>
-      <c r="C695" t="inlineStr">
+      <c r="C695" s="0" t="inlineStr">
         <is>
           <t>Recognise the truth about something — Calar.</t>
         </is>
       </c>
-      <c r="D695" t="inlineStr">
+      <c r="D695" s="0" t="inlineStr">
         <is>
           <t>Emma saw through the excuse.</t>
         </is>
       </c>
-      <c r="I695" t="inlineStr">
+      <c r="I695" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: see through — Present: sees through — Past: saw through — Past participle: seen through. Not separable in this sense.</t>
         </is>
       </c>
     </row>
     <row r="696">
-      <c r="A696" t="inlineStr">
+      <c r="A696" s="0" t="inlineStr">
         <is>
           <t>Stand up for</t>
         </is>
       </c>
-      <c r="B696" t="inlineStr">
+      <c r="B696" s="0" t="inlineStr">
         <is>
           <t>stand ap for</t>
         </is>
       </c>
-      <c r="C696" t="inlineStr">
+      <c r="C696" s="0" t="inlineStr">
         <is>
           <t>Defend someone or something — Defender.</t>
         </is>
       </c>
-      <c r="D696" t="inlineStr">
+      <c r="D696" s="0" t="inlineStr">
         <is>
           <t>Jack stood up for his friend.</t>
         </is>
       </c>
-      <c r="I696" t="inlineStr">
+      <c r="I696" s="0" t="inlineStr">
         <is>
           <t>Irregular verb. Base: stand up for — Present: stands up for — Past: stood up for — Past participle: stood up for. Not separable.</t>
         </is>

</xml_diff>

<commit_message>
Say the right version back, and be told whether you did
Reading a correction and moving on is how the same mistake arrives again
in the next sentence. So every correction now carries a button that
reads the right version out loud, listens for it to be repeated, and
marks the result word by word -- green for what was said, underlined for
what was missed, with a score and an invitation to go again.

It uses the scoring the speaking cards already had, so "I am going" said
in place of "I went" comes back as fifty per cent with the wrong word
marked, rather than a pass.

While talking, the correction sits beside the circle and practising it
borrows the microphone from the conversation, then gives it back: the
conversation is listening again the moment the repeat is scored. Two
things listening at once would mean neither heard anything, which is
what made this worth doing carefully rather than quickly.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I713"/>
+  <dimension ref="A1:I714"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col width="18.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -24826,29 +24826,51 @@
       </c>
     </row>
     <row r="713">
-      <c r="A713" t="inlineStr">
+      <c r="A713" s="0" t="inlineStr">
         <is>
           <t>Drive on up</t>
         </is>
       </c>
-      <c r="B713" t="inlineStr">
+      <c r="B713" s="0" t="inlineStr">
         <is>
           <t>draiv on ap</t>
         </is>
       </c>
-      <c r="C713" t="inlineStr">
+      <c r="C713" s="0" t="inlineStr">
         <is>
           <t>Move a vehicle closer by driving — Acercarse en vehículo.</t>
         </is>
       </c>
-      <c r="D713" t="inlineStr">
+      <c r="D713" s="0" t="inlineStr">
         <is>
           <t>Drive on up to the window.</t>
         </is>
       </c>
-      <c r="I713" t="inlineStr">
+      <c r="I713" s="0" t="inlineStr">
         <is>
           <t>Phrasal verb. Base: drive on up — Present: drives on up — Past: drove on up — Past participle: driven on up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Equator</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>ekuator</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Imaginary line around the middle of the Earth — Ecuador.</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>The equator divides the Earth into the Northern and Southern Hemispheres.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Start the hour again when ten new words arrive
The hour counted from the day the set arrived, which meant the time
spent that morning on the ten he already had was handed to the ten that
replaced them that afternoon. New words want their own hour.

So the moment a set is built, the clock reading is written down with it,
and the hour is the distance travelled since. Every second ever studied
only goes up -- the server refuses a write that would shorten a day --
so it serves as an odometer.

The set he is on now has no such mark, and counting it the new way would
take back thirty-four minutes he has already earned. It keeps the old
reckoning; the reset starts with his next ten.

Thirteen cases checked against the shipped code, with the date pinned
after the first run of them collided with the real one and passed two
tests for the wrong reason.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I717"/>
+  <dimension ref="A1:I728"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col width="18.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -24939,29 +24939,336 @@
       </c>
     </row>
     <row r="717">
-      <c r="A717" t="inlineStr">
+      <c r="A717" s="0" t="inlineStr">
         <is>
           <t>Shelves</t>
         </is>
       </c>
-      <c r="B717" t="inlineStr">
+      <c r="B717" s="0" t="inlineStr">
         <is>
           <t>ʃelvz</t>
         </is>
       </c>
-      <c r="C717" t="inlineStr">
+      <c r="C717" s="0" t="inlineStr">
         <is>
           <t>Horizontal boards for storage — Estantes.</t>
         </is>
       </c>
-      <c r="D717" t="inlineStr">
+      <c r="D717" s="0" t="inlineStr">
         <is>
           <t>The books are on the top shelves.</t>
         </is>
       </c>
-      <c r="I717" t="inlineStr">
+      <c r="I717" s="0" t="inlineStr">
         <is>
           <t>Plural of shelf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="0" t="inlineStr">
+        <is>
+          <t>Plenty</t>
+        </is>
+      </c>
+      <c r="B718" s="0" t="inlineStr">
+        <is>
+          <t>plenti</t>
+        </is>
+      </c>
+      <c r="C718" s="0" t="inlineStr">
+        <is>
+          <t>A large amount or quantity; more than enough — Abundancia, mucho.</t>
+        </is>
+      </c>
+      <c r="D718" s="0" t="inlineStr">
+        <is>
+          <t>We have plenty of food for the party.</t>
+        </is>
+      </c>
+      <c r="I718" s="0" t="inlineStr">
+        <is>
+          <t>Often followed by 'of'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="0" t="inlineStr">
+        <is>
+          <t>Shelf</t>
+        </is>
+      </c>
+      <c r="B719" s="0" t="inlineStr">
+        <is>
+          <t>chelf</t>
+        </is>
+      </c>
+      <c r="C719" s="0" t="inlineStr">
+        <is>
+          <t>A flat board fixed to a wall or inside a cupboard for holding things — Estante.</t>
+        </is>
+      </c>
+      <c r="D719" s="0" t="inlineStr">
+        <is>
+          <t>The book was on the top shelf.</t>
+        </is>
+      </c>
+      <c r="I719" s="0" t="inlineStr">
+        <is>
+          <t>Plural: shelves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="0" t="inlineStr">
+        <is>
+          <t>Trout</t>
+        </is>
+      </c>
+      <c r="B720" s="0" t="inlineStr">
+        <is>
+          <t>traut</t>
+        </is>
+      </c>
+      <c r="C720" s="0" t="inlineStr">
+        <is>
+          <t>Freshwater fish with a speckled body — Trucha.</t>
+        </is>
+      </c>
+      <c r="D720" s="0" t="inlineStr">
+        <is>
+          <t>We caught a big trout in the river.</t>
+        </is>
+      </c>
+      <c r="I720" s="0" t="inlineStr">
+        <is>
+          <t>Plural is usually trout, though trouts is sometimes used for different species.</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="0" t="inlineStr">
+        <is>
+          <t>Proudly</t>
+        </is>
+      </c>
+      <c r="B721" s="0" t="inlineStr">
+        <is>
+          <t>praudli</t>
+        </is>
+      </c>
+      <c r="C721" s="0" t="inlineStr">
+        <is>
+          <t>With pride — Con orgullo.</t>
+        </is>
+      </c>
+      <c r="D721" s="0" t="inlineStr">
+        <is>
+          <t>She proudly displayed her diploma.</t>
+        </is>
+      </c>
+      <c r="I721" s="0" t="inlineStr">
+        <is>
+          <t>Adverb formed from the adjective proud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="0" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="B722" s="0" t="inlineStr">
+        <is>
+          <t>kleim</t>
+        </is>
+      </c>
+      <c r="C722" s="0" t="inlineStr">
+        <is>
+          <t>State that something is the case, typically without providing evidence — Afirmar, asegurar.</t>
+        </is>
+      </c>
+      <c r="D722" s="0" t="inlineStr">
+        <is>
+          <t>He claims that he saw the ghost.</t>
+        </is>
+      </c>
+      <c r="E722" s="0" t="inlineStr">
+        <is>
+          <t>Formally request or demand something because you believe you have a right to it — Reclamar, exigir.</t>
+        </is>
+      </c>
+      <c r="F722" s="0" t="inlineStr">
+        <is>
+          <t>You can claim your money back.</t>
+        </is>
+      </c>
+      <c r="I722" s="0" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: claim — Present: claims — Past: claimed — Past participle: claimed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="0" t="inlineStr">
+        <is>
+          <t>Shimmering</t>
+        </is>
+      </c>
+      <c r="B723" s="0" t="inlineStr">
+        <is>
+          <t>shímering</t>
+        </is>
+      </c>
+      <c r="C723" s="0" t="inlineStr">
+        <is>
+          <t>Reflecting a soft, tremulous light — Brillante o trémulo.</t>
+        </is>
+      </c>
+      <c r="D723" s="0" t="inlineStr">
+        <is>
+          <t>The shimmering surface of the lake looked magical.</t>
+        </is>
+      </c>
+      <c r="I723" s="0" t="inlineStr">
+        <is>
+          <t>Present participle/adjective formed from the verb shimmer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="0" t="inlineStr">
+        <is>
+          <t>Stretches</t>
+        </is>
+      </c>
+      <c r="B724" s="0" t="inlineStr">
+        <is>
+          <t>stréchis</t>
+        </is>
+      </c>
+      <c r="C724" s="0" t="inlineStr">
+        <is>
+          <t>Extends or pulls something so that it becomes longer or wider — Estira.</t>
+        </is>
+      </c>
+      <c r="D724" s="0" t="inlineStr">
+        <is>
+          <t>She stretches her legs before running.</t>
+        </is>
+      </c>
+      <c r="I724" s="0" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: stretch — Present: stretches — Past: stretched — Past participle: stretched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="0" t="inlineStr">
+        <is>
+          <t>Joggers</t>
+        </is>
+      </c>
+      <c r="B725" s="0" t="inlineStr">
+        <is>
+          <t>yóguers</t>
+        </is>
+      </c>
+      <c r="C725" s="0" t="inlineStr">
+        <is>
+          <t>Soft, loose trousers worn for exercise or relaxing — Pantalones de chándal.</t>
+        </is>
+      </c>
+      <c r="D725" s="0" t="inlineStr">
+        <is>
+          <t>He put on a t-shirt and joggers.</t>
+        </is>
+      </c>
+      <c r="I725" s="0" t="inlineStr">
+        <is>
+          <t>Plural noun. Always used in the plural for this meaning (singular 'jogger' refers to a person who runs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="0" t="inlineStr">
+        <is>
+          <t>Jogger</t>
+        </is>
+      </c>
+      <c r="B726" s="0" t="inlineStr">
+        <is>
+          <t>yóguer</t>
+        </is>
+      </c>
+      <c r="C726" s="0" t="inlineStr">
+        <is>
+          <t>Person who runs for exercise — Corredor (que hace footing).</t>
+        </is>
+      </c>
+      <c r="D726" s="0" t="inlineStr">
+        <is>
+          <t>A jogger ran past our house.</t>
+        </is>
+      </c>
+      <c r="I726" s="0" t="inlineStr">
+        <is>
+          <t>Usually refers to recreational runners rather than competitive ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="0" t="inlineStr">
+        <is>
+          <t>Effortless</t>
+        </is>
+      </c>
+      <c r="B727" s="0" t="inlineStr">
+        <is>
+          <t>éf-ort-les</t>
+        </is>
+      </c>
+      <c r="C727" s="0" t="inlineStr">
+        <is>
+          <t>Requiring no physical or mental exertion — Sin esfuerzo.</t>
+        </is>
+      </c>
+      <c r="D727" s="0" t="inlineStr">
+        <is>
+          <t>Her performance on the piano looked completely effortless.</t>
+        </is>
+      </c>
+      <c r="I727" s="0" t="inlineStr">
+        <is>
+          <t>Adjective. Often used to describe skills, beauty, or movement that seems natural and easy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Beauty</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>biuti</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>The quality of being pleasing or attractive — Belleza.</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>She admires the natural beauty of the mountains.</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>Countable noun when referring to a beautiful person or thing (e.g., 'She was a beauty in her youth').</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep the words he added while I was testing
The spreadsheet moved under me during the test pass -- he has been
adding words -- so the file is committed as it stands, with my own test
word taken back out of it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -25246,27 +25246,27 @@
       </c>
     </row>
     <row r="728">
-      <c r="A728" t="inlineStr">
+      <c r="A728" s="0" t="inlineStr">
         <is>
           <t>Beauty</t>
         </is>
       </c>
-      <c r="B728" t="inlineStr">
+      <c r="B728" s="0" t="inlineStr">
         <is>
           <t>biuti</t>
         </is>
       </c>
-      <c r="C728" t="inlineStr">
+      <c r="C728" s="0" t="inlineStr">
         <is>
           <t>The quality of being pleasing or attractive — Belleza.</t>
         </is>
       </c>
-      <c r="D728" t="inlineStr">
+      <c r="D728" s="0" t="inlineStr">
         <is>
           <t>She admires the natural beauty of the mountains.</t>
         </is>
       </c>
-      <c r="I728" t="inlineStr">
+      <c r="I728" s="0" t="inlineStr">
         <is>
           <t>Countable noun when referring to a beautiful person or thing (e.g., 'She was a beauty in her youth').</t>
         </is>

</xml_diff>

<commit_message>
A conversation that does not have to be earned
The day's conversation opens when the day's ten are mastered, which is
right for the day's ten and wrong for nine o'clock at night when he
wants to talk. So there is a second way in, always there: the same
partner, the same situations, the same corrections, on ten words he has
already mastered -- the ones longest since he last saw them, because a
word he can recognise on a card and cannot reach for in a sentence is
not yet his.

Nothing in it is counted. It does not touch the day's set, the hour, or
the gate.

The ten are chosen once and held. Building a situation redraws the
picker, and the first version reshuffled on every redraw -- so the
situation was invented for one set of words and the conversation then
ran on another, which is how a sentence with Tapes in it could tick
nothing: Tapes was no longer one of the ten by then.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I728"/>
+  <dimension ref="A1:I730"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col width="18.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -25269,6 +25269,60 @@
       <c r="I728" s="0" t="inlineStr">
         <is>
           <t>Countable noun when referring to a beautiful person or thing (e.g., 'She was a beauty in her youth').</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="0" t="inlineStr">
+        <is>
+          <t>Detached</t>
+        </is>
+      </c>
+      <c r="B729" s="0" t="inlineStr">
+        <is>
+          <t>ditácht</t>
+        </is>
+      </c>
+      <c r="C729" s="0" t="inlineStr">
+        <is>
+          <t>Not connected or separate — Separado / independiente.</t>
+        </is>
+      </c>
+      <c r="D729" s="0" t="inlineStr">
+        <is>
+          <t>The house has a detached garage.</t>
+        </is>
+      </c>
+      <c r="I729" s="0" t="inlineStr">
+        <is>
+          <t>Often used to describe houses that are not joined to another property, or a person who is emotionally removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Handle</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>jándel</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Part of something designed to be held or opened by — Manija / mango / tirador.</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>The handle of the suitcase broke.</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>Regular verb. Base: handle — Present: handles — Past: handled — Past participle: handled. Also used as a noun.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Free talk does not buy the next ten words
He noticed the bar climbing while he was talking freely, and he is
right: the hour exists to be paid in the ten words he has, and an
evening spent chatting with words he mastered a fortnight ago is worth
doing and is not that. The clock now stops for a practice conversation
and runs for everything else -- cards, the check at the door, and the
day's own conversation. Eight cases checked against the shipped code.

And a way to put the figure right when it is wrong, under the bar: start
this hour again, which asks before it does anything and then sets the
mark to here. It moves only what counts toward the current ten. The
record of what was studied is not touched, so the calendar and the
history are unchanged -- a reset of the clock is not a confession that
the time was never spent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I764"/>
+  <dimension ref="A1:I765"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col width="18.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -26243,29 +26243,56 @@
       </c>
     </row>
     <row r="764">
-      <c r="A764" t="inlineStr">
+      <c r="A764" s="0" t="inlineStr">
         <is>
           <t>Forward</t>
         </is>
       </c>
-      <c r="B764" t="inlineStr">
+      <c r="B764" s="0" t="inlineStr">
         <is>
           <t>fórward</t>
         </is>
       </c>
-      <c r="C764" t="inlineStr">
+      <c r="C764" s="0" t="inlineStr">
         <is>
           <t>Proceed or progress with an action or plan — Seguir adelante.</t>
         </is>
       </c>
-      <c r="D764" t="inlineStr">
+      <c r="D764" s="0" t="inlineStr">
         <is>
           <t>Are we good to move forward with that plan?</t>
         </is>
       </c>
-      <c r="I764" t="inlineStr">
+      <c r="I764" s="0" t="inlineStr">
         <is>
           <t>Often used with verbs like 'move', 'go', or 'press'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>How are you keeping</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>jau ar yu ki-ping</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>How are you? — ¿Cómo estás? o ¿Cómo te va?</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Hello, John! How are you keeping?</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>Informal greeting used mainly in British English to ask about someone's health or general well-being over a period of time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Escape leaves the check at the door
Ten words is the right thing to be asked and the wrong thing to be
trapped by: opening the app to do something else should not mean
answering your way past it first.

Escape closes it from anywhere in the run -- the typing box, the answer
panel, the summary -- and from wherever the focus happens to be, since
the panel only hears the key when something inside it is focused and
"almost always" is no use to somebody holding Escape down. The way out
on screen says Esc now, so it can be found without being told.

What was already answered is kept; the rest is simply not asked.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ENGLISH SCHOOL.xlsx
+++ b/ENGLISH SCHOOL.xlsx
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I767"/>
+  <dimension ref="A1:I768"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col width="18.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -26334,29 +26334,56 @@
       </c>
     </row>
     <row r="767">
-      <c r="A767" t="inlineStr">
+      <c r="A767" s="0" t="inlineStr">
         <is>
           <t>Adulthood</t>
         </is>
       </c>
-      <c r="B767" t="inlineStr">
+      <c r="B767" s="0" t="inlineStr">
         <is>
           <t>aduljud</t>
         </is>
       </c>
-      <c r="C767" t="inlineStr">
+      <c r="C767" s="0" t="inlineStr">
         <is>
           <t>The state or condition of being a adult — Edad adulta.</t>
         </is>
       </c>
-      <c r="D767" t="inlineStr">
+      <c r="D767" s="0" t="inlineStr">
         <is>
           <t>He reached adulthood at eighteen.</t>
         </is>
       </c>
-      <c r="I767" t="inlineStr">
+      <c r="I767" s="0" t="inlineStr">
         <is>
           <t>Noun.</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>Thoughtfully</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>zótfuli</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>In a quiet, deep, or considerate way — Pensativamente / Con consideración.</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>He looked at the painting thoughtfully before speaking.</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>Adverb. Derived from the adjective 'thoughtful'.</t>
         </is>
       </c>
     </row>

</xml_diff>